<commit_message>
docs: ajusta tres fases de laboratorio tras la revision final por entregable
</commit_message>
<xml_diff>
--- a/docs/requerimientos-entrega.xlsx
+++ b/docs/requerimientos-entrega.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\roomtrip\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{791BE8E4-2522-4CF1-A1FF-8A25A3A25A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A136C917-9A6F-4BC3-852B-379461026AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="195" windowWidth="21600" windowHeight="15405" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="195" windowWidth="21600" windowHeight="15405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="224">
   <si>
     <t>RoomTrip</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t>1TEL05 — Servicios y Aplicaciones para IoT</t>
+  </si>
+  <si>
+    <t>Carrera</t>
+  </si>
+  <si>
+    <t>Ingeniería de las Telecomunicaciones — PUCP</t>
   </si>
   <si>
     <t>Semestre</t>
@@ -825,7 +831,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -848,37 +854,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCFD8DC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCFD8DC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCFD8DC"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFCFD8DC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -962,18 +942,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1039,7 +1007,6 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="es-PE"/>
               <a:t>Requerimientos por rol</a:t>
             </a:r>
           </a:p>
@@ -1123,7 +1090,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8213-4680-95CB-0748E5B647CD}"/>
+              <c16:uniqueId val="{00000000-83CA-4BFD-9357-45BEAC01379F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1175,7 +1142,6 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="es-PE"/>
                   <a:t>Cantidad</a:t>
                 </a:r>
               </a:p>
@@ -1559,34 +1525,38 @@
       <c r="D5" s="27"/>
     </row>
     <row r="6" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="38"/>
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>0</v>
@@ -1596,27 +1566,27 @@
     </row>
     <row r="10" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="3"/>
@@ -1624,7 +1594,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B13" s="29"/>
       <c r="C13" s="29"/>
@@ -1632,7 +1602,7 @@
     </row>
     <row r="15" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15" s="27"/>
       <c r="C15" s="27"/>
@@ -1640,7 +1610,7 @@
     </row>
     <row r="16" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="28" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B16" s="29"/>
       <c r="C16" s="29"/>
@@ -1648,7 +1618,7 @@
     </row>
     <row r="17" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="28" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B17" s="29"/>
       <c r="C17" s="29"/>
@@ -1656,7 +1626,7 @@
     </row>
     <row r="18" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="28" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" s="29"/>
       <c r="C18" s="29"/>
@@ -1664,7 +1634,7 @@
     </row>
     <row r="20" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B20" s="27"/>
       <c r="C20" s="27"/>
@@ -1672,47 +1642,47 @@
     </row>
     <row r="21" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
     </row>
     <row r="23" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
     </row>
     <row r="24" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
     </row>
     <row r="26" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="26" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
@@ -1720,7 +1690,7 @@
     </row>
     <row r="27" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B27" s="29"/>
       <c r="C27" s="29"/>
@@ -1728,7 +1698,7 @@
     </row>
     <row r="28" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="30" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B28" s="29"/>
       <c r="C28" s="29"/>
@@ -1736,7 +1706,7 @@
     </row>
     <row r="29" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="30" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B29" s="29"/>
       <c r="C29" s="29"/>
@@ -1744,7 +1714,7 @@
     </row>
     <row r="30" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="30" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B30" s="29"/>
       <c r="C30" s="29"/>
@@ -1752,7 +1722,7 @@
     </row>
     <row r="31" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="30" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B31" s="29"/>
       <c r="C31" s="29"/>
@@ -1760,18 +1730,16 @@
     </row>
     <row r="32" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="30" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B32" s="29"/>
       <c r="C32" s="29"/>
       <c r="D32" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="16">
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="A26:D26"/>
@@ -1788,7 +1756,6 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1803,7 +1770,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -1813,7 +1780,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -1823,7 +1790,7 @@
     </row>
     <row r="3" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
@@ -1833,7 +1800,7 @@
     </row>
     <row r="5" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="27"/>
@@ -1843,22 +1810,22 @@
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
@@ -1888,7 +1855,7 @@
     </row>
     <row r="9" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B9" s="27"/>
       <c r="C9" s="27"/>
@@ -1898,27 +1865,27 @@
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B11" s="11">
         <f>COUNTIF(Requerimientos!$C$6:$C$52,$A11)</f>
@@ -1943,7 +1910,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B12" s="13">
         <f>COUNTIF(Requerimientos!$C$6:$C$52,$A12)</f>
@@ -1968,7 +1935,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" s="11">
         <f>COUNTIF(Requerimientos!$C$6:$C$52,$A13)</f>
@@ -1993,7 +1960,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B14" s="13">
         <f>COUNTIF(Requerimientos!$C$6:$C$52,$A14)</f>
@@ -2018,7 +1985,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B15" s="11">
         <f>COUNTIF(Requerimientos!$C$6:$C$52,$A15)</f>
@@ -2043,7 +2010,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B16" s="15">
         <f>SUM(B11:B15)</f>
@@ -2068,7 +2035,7 @@
     </row>
     <row r="18" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B18" s="27"/>
       <c r="C18" s="27"/>
@@ -2078,27 +2045,27 @@
     </row>
     <row r="19" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B20" s="13">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A20)</f>
@@ -2123,7 +2090,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B21" s="11">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A21)</f>
@@ -2148,7 +2115,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B22" s="13">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A22)</f>
@@ -2173,7 +2140,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B23" s="11">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A23)</f>
@@ -2198,7 +2165,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B24" s="13">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A24)</f>
@@ -2223,7 +2190,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B25" s="11">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A25)</f>
@@ -2248,7 +2215,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B26" s="13">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A26)</f>
@@ -2273,7 +2240,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B27" s="11">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A27)</f>
@@ -2298,7 +2265,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B28" s="13">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A28)</f>
@@ -2323,7 +2290,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B29" s="11">
         <f>COUNTIF(Requerimientos!$B$6:$B$52,$A29)</f>
@@ -2348,7 +2315,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B30" s="15">
         <f>SUM(B20:B29)</f>
@@ -2404,7 +2371,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -2415,7 +2382,7 @@
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -2426,7 +2393,7 @@
     </row>
     <row r="3" spans="1:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
@@ -2437,1106 +2404,1106 @@
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="18" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E16" s="19" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C17" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="G17" s="23" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="F17" s="22" t="s">
-        <v>108</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C18" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" s="20" t="s">
         <v>49</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>111</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C20" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="F20" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="G20" s="20" t="s">
         <v>49</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="G20" s="20" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G28" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F29" s="22" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="18" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G30" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="18" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E36" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G40" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D42" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G42" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F43" s="22" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E44" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G44" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F45" s="22" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G46" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F47" s="22" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="18" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G48" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F49" s="22" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="18" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D50" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G50" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B51" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F51" s="22" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="18" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G52" s="20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -3577,7 +3544,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -3587,7 +3554,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="31" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -3597,7 +3564,7 @@
     </row>
     <row r="3" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
@@ -3607,27 +3574,27 @@
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>68</v>
-      </c>
       <c r="F5" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
@@ -3637,107 +3604,107 @@
     </row>
     <row r="7" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -3747,207 +3714,207 @@
     </row>
     <row r="14" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="26" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B25" s="27"/>
       <c r="C25" s="27"/>
@@ -3957,147 +3924,147 @@
     </row>
     <row r="26" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B27" s="22" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="26" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
@@ -4107,247 +4074,247 @@
     </row>
     <row r="35" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B38" s="22" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B40" s="22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B42" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B46" s="22" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F46" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="26" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B48" s="27"/>
       <c r="C48" s="27"/>
@@ -4357,262 +4324,262 @@
     </row>
     <row r="49" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B49" s="22" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C49" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E49" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="D49" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E49" s="23" t="s">
-        <v>176</v>
-      </c>
       <c r="F49" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B50" s="22" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B51" s="22" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B52" s="22" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E52" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F52" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B53" s="22" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E53" s="23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F53" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B54" s="22" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E54" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F54" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="21" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B55" s="22" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E55" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F55" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="21" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E56" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F56" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B57" s="22" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E57" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F57" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="21" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E58" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F58" s="23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="21" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E59" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F59" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="21" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B60" s="22" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E60" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F60" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="21" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B61" s="22" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E61" s="23" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F61" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: excluye los dos requerimientos derivados de la version de entrega y precisa el criterio de RF-CL-01
</commit_message>
<xml_diff>
--- a/docs/requerimientos-entrega.xlsx
+++ b/docs/requerimientos-entrega.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\roomtrip\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A136C917-9A6F-4BC3-852B-379461026AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCEFFA47-2D85-4059-AF59-A348F0E04D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="390" yWindow="195" windowWidth="21600" windowHeight="15405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Por rol" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Requerimientos!$A$5:$G$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Requerimientos!$A$5:$G$50</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por rol'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">Requerimientos!$5:$5</definedName>
   </definedNames>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="218">
   <si>
     <t>RoomTrip</t>
   </si>
@@ -355,15 +355,6 @@
     <t>El hotel ve solo los chats de reservas activas y puede responder</t>
   </si>
   <si>
-    <t>RF-AH-10</t>
-  </si>
-  <si>
-    <t>Establecer el monto mínimo de reserva que da derecho al taxi gratuito al aeropuerto</t>
-  </si>
-  <si>
-    <t>El hotel guarda un monto mínimo y solo las reservas que lo alcanzan habilitan la opción de taxi al cliente</t>
-  </si>
-  <si>
     <t>RF-AH-07</t>
   </si>
   <si>
@@ -469,7 +460,7 @@
     <t>Autoregistrarse y quedar habilitado automáticamente</t>
   </si>
   <si>
-    <t>Al completar el formulario con nombres apellidos tipo y número de documento fecha de nacimiento correo teléfono domicilio y foto la cuenta queda activa sin aprobación</t>
+    <t>Al completar el formulario con nombres, apellidos, tipo de documento (DNI, Pasaporte o Carnet de extranjería), número de documento, fecha de nacimiento, correo, teléfono, domicilio y foto, la cuenta queda activa sin necesidad de aprobación</t>
   </si>
   <si>
     <t>RF-CL-02</t>
@@ -526,15 +517,6 @@
     <t>El historial lista las reservas del cliente autenticado con fechas hotel habitación estado y monto</t>
   </si>
   <si>
-    <t>RF-CL-12</t>
-  </si>
-  <si>
-    <t>Consultar los lugares históricos cercanos al hotel</t>
-  </si>
-  <si>
-    <t>El cliente ve la lista de lugares históricos cercanos registrados por el administrador del hotel</t>
-  </si>
-  <si>
     <t>RF-CL-08</t>
   </si>
   <si>
@@ -700,13 +682,13 @@
     <t>Superadmin    ·    5 requerimientos</t>
   </si>
   <si>
-    <t>Administrador de hotel    ·    10 requerimientos</t>
+    <t>Administrador de hotel    ·    9 requerimientos</t>
   </si>
   <si>
     <t>Taxista    ·    7 requerimientos</t>
   </si>
   <si>
-    <t>Cliente    ·    12 requerimientos</t>
+    <t>Cliente    ·    11 requerimientos</t>
   </si>
   <si>
     <t>Transversal    ·    13 requerimientos</t>
@@ -1074,13 +1056,13 @@
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>12</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>13</c:v>
@@ -1090,7 +1072,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-83CA-4BFD-9357-45BEAC01379F}"/>
+              <c16:uniqueId val="{00000000-C17C-4CB8-953E-3BE1694A13F1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1830,24 +1812,24 @@
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
-        <f>COUNTA(Requerimientos!$A$6:$A$52)</f>
-        <v>47</v>
+        <f>COUNTA(Requerimientos!$A$6:$A$50)</f>
+        <v>45</v>
       </c>
       <c r="B7" s="9">
-        <f>COUNTIF(Requerimientos!$D$6:$D$52,"Funcional")</f>
-        <v>38</v>
+        <f>COUNTIF(Requerimientos!$D$6:$D$50,"Funcional")</f>
+        <v>36</v>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIF(Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIF(Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>9</v>
       </c>
       <c r="D7" s="9">
-        <f>COUNTIF(Requerimientos!$G$6:$G$52,"Alta")</f>
-        <v>38</v>
+        <f>COUNTIF(Requerimientos!$G$6:$G$50,"Alta")</f>
+        <v>37</v>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIF(Requerimientos!$G$6:$G$52,"Media")</f>
-        <v>9</v>
+        <f>COUNTIF(Requerimientos!$G$6:$G$50,"Media")</f>
+        <v>8</v>
       </c>
       <c r="F7" s="9">
         <v>10</v>
@@ -1888,23 +1870,23 @@
         <v>50</v>
       </c>
       <c r="B11" s="11">
-        <f>COUNTIF(Requerimientos!$C$6:$C$52,$A11)</f>
+        <f>COUNTIF(Requerimientos!$C$6:$C$50,$A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A11,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A11,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>5</v>
       </c>
       <c r="D11" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A11,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A11,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E11" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A11,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A11,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>3</v>
       </c>
       <c r="F11" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A11,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A11,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>2</v>
       </c>
     </row>
@@ -1913,23 +1895,23 @@
         <v>51</v>
       </c>
       <c r="B12" s="13">
-        <f>COUNTIF(Requerimientos!$C$6:$C$52,$A12)</f>
-        <v>10</v>
+        <f>COUNTIF(Requerimientos!$C$6:$C$50,$A12)</f>
+        <v>9</v>
       </c>
       <c r="C12" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A12,Requerimientos!$D$6:$D$52,"Funcional")</f>
-        <v>10</v>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A12,Requerimientos!$D$6:$D$50,"Funcional")</f>
+        <v>9</v>
       </c>
       <c r="D12" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A12,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A12,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E12" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A12,Requerimientos!$G$6:$G$52,"Alta")</f>
-        <v>7</v>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A12,Requerimientos!$G$6:$G$50,"Alta")</f>
+        <v>6</v>
       </c>
       <c r="F12" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A12,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A12,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>3</v>
       </c>
     </row>
@@ -1938,23 +1920,23 @@
         <v>52</v>
       </c>
       <c r="B13" s="11">
-        <f>COUNTIF(Requerimientos!$C$6:$C$52,$A13)</f>
+        <f>COUNTIF(Requerimientos!$C$6:$C$50,$A13)</f>
         <v>7</v>
       </c>
       <c r="C13" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A13,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A13,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>7</v>
       </c>
       <c r="D13" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A13,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A13,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E13" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A13,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A13,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>7</v>
       </c>
       <c r="F13" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A13,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A13,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>0</v>
       </c>
     </row>
@@ -1963,24 +1945,24 @@
         <v>53</v>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIF(Requerimientos!$C$6:$C$52,$A14)</f>
-        <v>12</v>
+        <f>COUNTIF(Requerimientos!$C$6:$C$50,$A14)</f>
+        <v>11</v>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A14,Requerimientos!$D$6:$D$52,"Funcional")</f>
-        <v>12</v>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A14,Requerimientos!$D$6:$D$50,"Funcional")</f>
+        <v>11</v>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A14,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A14,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E14" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A14,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A14,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>9</v>
       </c>
       <c r="F14" s="13">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A14,Requerimientos!$G$6:$G$52,"Media")</f>
-        <v>3</v>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A14,Requerimientos!$G$6:$G$50,"Media")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1988,23 +1970,23 @@
         <v>54</v>
       </c>
       <c r="B15" s="11">
-        <f>COUNTIF(Requerimientos!$C$6:$C$52,$A15)</f>
+        <f>COUNTIF(Requerimientos!$C$6:$C$50,$A15)</f>
         <v>13</v>
       </c>
       <c r="C15" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A15,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A15,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>4</v>
       </c>
       <c r="D15" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A15,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A15,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>9</v>
       </c>
       <c r="E15" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A15,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A15,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>12</v>
       </c>
       <c r="F15" s="11">
-        <f>COUNTIFS(Requerimientos!$C$6:$C$52,$A15,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$C$6:$C$50,$A15,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>1</v>
       </c>
     </row>
@@ -2014,11 +1996,11 @@
       </c>
       <c r="B16" s="15">
         <f>SUM(B11:B15)</f>
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C16" s="15">
         <f>SUM(C11:C15)</f>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D16" s="15">
         <f>SUM(D11:D15)</f>
@@ -2026,11 +2008,11 @@
       </c>
       <c r="E16" s="15">
         <f>SUM(E11:E15)</f>
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F11:F15)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -2068,23 +2050,23 @@
         <v>57</v>
       </c>
       <c r="B20" s="13">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A20)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A20)</f>
         <v>4</v>
       </c>
       <c r="C20" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A20,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A20,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>4</v>
       </c>
       <c r="D20" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A20,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A20,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E20" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A20,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A20,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>4</v>
       </c>
       <c r="F20" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A20,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A20,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>0</v>
       </c>
     </row>
@@ -2093,23 +2075,23 @@
         <v>58</v>
       </c>
       <c r="B21" s="11">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A21)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A21)</f>
         <v>3</v>
       </c>
       <c r="C21" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A21,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A21,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>3</v>
       </c>
       <c r="D21" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A21,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A21,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E21" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A21,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A21,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>3</v>
       </c>
       <c r="F21" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A21,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A21,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>0</v>
       </c>
     </row>
@@ -2118,24 +2100,24 @@
         <v>59</v>
       </c>
       <c r="B22" s="13">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A22)</f>
-        <v>6</v>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A22)</f>
+        <v>5</v>
       </c>
       <c r="C22" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A22,Requerimientos!$D$6:$D$52,"Funcional")</f>
-        <v>6</v>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A22,Requerimientos!$D$6:$D$50,"Funcional")</f>
+        <v>5</v>
       </c>
       <c r="D22" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A22,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A22,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E22" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A22,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A22,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>5</v>
       </c>
       <c r="F22" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A22,Requerimientos!$G$6:$G$52,"Media")</f>
-        <v>1</v>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A22,Requerimientos!$G$6:$G$50,"Media")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2143,23 +2125,23 @@
         <v>60</v>
       </c>
       <c r="B23" s="11">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A23)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A23)</f>
         <v>4</v>
       </c>
       <c r="C23" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A23,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A23,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>4</v>
       </c>
       <c r="D23" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A23,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A23,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E23" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A23,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A23,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>3</v>
       </c>
       <c r="F23" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A23,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A23,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>1</v>
       </c>
     </row>
@@ -2168,23 +2150,23 @@
         <v>61</v>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A24)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A24)</f>
         <v>3</v>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A24,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A24,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>3</v>
       </c>
       <c r="D24" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A24,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A24,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E24" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A24,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A24,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>2</v>
       </c>
       <c r="F24" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A24,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A24,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>1</v>
       </c>
     </row>
@@ -2193,23 +2175,23 @@
         <v>62</v>
       </c>
       <c r="B25" s="11">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A25)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A25)</f>
         <v>1</v>
       </c>
       <c r="C25" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A25,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A25,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>1</v>
       </c>
       <c r="D25" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A25,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A25,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E25" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A25,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A25,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>1</v>
       </c>
       <c r="F25" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A25,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A25,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>0</v>
       </c>
     </row>
@@ -2218,23 +2200,23 @@
         <v>63</v>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A26)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A26)</f>
         <v>3</v>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A26,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A26,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>3</v>
       </c>
       <c r="D26" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A26,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A26,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E26" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A26,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A26,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>3</v>
       </c>
       <c r="F26" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A26,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A26,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>0</v>
       </c>
     </row>
@@ -2243,23 +2225,23 @@
         <v>64</v>
       </c>
       <c r="B27" s="11">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A27)</f>
-        <v>11</v>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A27)</f>
+        <v>10</v>
       </c>
       <c r="C27" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A27,Requerimientos!$D$6:$D$52,"Funcional")</f>
-        <v>11</v>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A27,Requerimientos!$D$6:$D$50,"Funcional")</f>
+        <v>10</v>
       </c>
       <c r="D27" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A27,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A27,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E27" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A27,Requerimientos!$G$6:$G$52,"Alta")</f>
-        <v>9</v>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A27,Requerimientos!$G$6:$G$50,"Alta")</f>
+        <v>8</v>
       </c>
       <c r="F27" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A27,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A27,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>2</v>
       </c>
     </row>
@@ -2268,23 +2250,23 @@
         <v>65</v>
       </c>
       <c r="B28" s="13">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A28)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A28)</f>
         <v>3</v>
       </c>
       <c r="C28" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A28,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A28,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>3</v>
       </c>
       <c r="D28" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A28,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A28,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>0</v>
       </c>
       <c r="E28" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A28,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A28,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>0</v>
       </c>
       <c r="F28" s="13">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A28,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A28,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>3</v>
       </c>
     </row>
@@ -2293,23 +2275,23 @@
         <v>66</v>
       </c>
       <c r="B29" s="11">
-        <f>COUNTIF(Requerimientos!$B$6:$B$52,$A29)</f>
+        <f>COUNTIF(Requerimientos!$B$6:$B$50,$A29)</f>
         <v>9</v>
       </c>
       <c r="C29" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A29,Requerimientos!$D$6:$D$52,"Funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A29,Requerimientos!$D$6:$D$50,"Funcional")</f>
         <v>0</v>
       </c>
       <c r="D29" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A29,Requerimientos!$D$6:$D$52,"No funcional")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A29,Requerimientos!$D$6:$D$50,"No funcional")</f>
         <v>9</v>
       </c>
       <c r="E29" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A29,Requerimientos!$G$6:$G$52,"Alta")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A29,Requerimientos!$G$6:$G$50,"Alta")</f>
         <v>8</v>
       </c>
       <c r="F29" s="11">
-        <f>COUNTIFS(Requerimientos!$B$6:$B$52,$A29,Requerimientos!$G$6:$G$52,"Media")</f>
+        <f>COUNTIFS(Requerimientos!$B$6:$B$50,$A29,Requerimientos!$G$6:$G$50,"Media")</f>
         <v>1</v>
       </c>
     </row>
@@ -2319,11 +2301,11 @@
       </c>
       <c r="B30" s="15">
         <f>SUM(B20:B29)</f>
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C30" s="15">
         <f>SUM(C20:C29)</f>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D30" s="15">
         <f>SUM(D20:D29)</f>
@@ -2331,11 +2313,11 @@
       </c>
       <c r="E30" s="15">
         <f>SUM(E20:E29)</f>
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F30" s="15">
         <f>SUM(F20:F29)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2357,7 +2339,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2660,7 +2642,7 @@
         <v>105</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C16" s="20" t="s">
         <v>51</v>
@@ -2675,7 +2657,7 @@
         <v>107</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2683,7 +2665,7 @@
         <v>108</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C17" s="23" t="s">
         <v>51</v>
@@ -2706,7 +2688,7 @@
         <v>111</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C18" s="20" t="s">
         <v>51</v>
@@ -2721,7 +2703,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2729,7 +2711,7 @@
         <v>114</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C19" s="23" t="s">
         <v>51</v>
@@ -2744,7 +2726,7 @@
         <v>116</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2752,10 +2734,10 @@
         <v>117</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>75</v>
@@ -2767,7 +2749,7 @@
         <v>119</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -2775,7 +2757,7 @@
         <v>120</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>52</v>
@@ -2890,7 +2872,7 @@
         <v>135</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C26" s="20" t="s">
         <v>52</v>
@@ -2916,7 +2898,7 @@
         <v>57</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D27" s="23" t="s">
         <v>75</v>
@@ -2936,7 +2918,7 @@
         <v>141</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C28" s="20" t="s">
         <v>53</v>
@@ -2959,7 +2941,7 @@
         <v>144</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>53</v>
@@ -2982,7 +2964,7 @@
         <v>147</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C30" s="20" t="s">
         <v>53</v>
@@ -3005,7 +2987,7 @@
         <v>150</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>53</v>
@@ -3028,7 +3010,7 @@
         <v>153</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C32" s="20" t="s">
         <v>53</v>
@@ -3051,7 +3033,7 @@
         <v>156</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>53</v>
@@ -3066,7 +3048,7 @@
         <v>158</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3074,7 +3056,7 @@
         <v>159</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C34" s="20" t="s">
         <v>53</v>
@@ -3089,7 +3071,7 @@
         <v>161</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3097,7 +3079,7 @@
         <v>162</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C35" s="23" t="s">
         <v>53</v>
@@ -3112,7 +3094,7 @@
         <v>164</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3158,7 +3140,7 @@
         <v>170</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3166,19 +3148,19 @@
         <v>171</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D38" s="20" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G38" s="20" t="s">
         <v>48</v>
@@ -3186,39 +3168,39 @@
     </row>
     <row r="39" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B39" s="22" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D39" s="23" t="s">
         <v>75</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C40" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>178</v>
+        <v>75</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>179</v>
@@ -3235,7 +3217,7 @@
         <v>181</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C41" s="23" t="s">
         <v>54</v>
@@ -3258,7 +3240,7 @@
         <v>184</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C42" s="20" t="s">
         <v>54</v>
@@ -3281,13 +3263,13 @@
         <v>187</v>
       </c>
       <c r="B43" s="22" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C43" s="23" t="s">
         <v>54</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="E43" s="22" t="s">
         <v>188</v>
@@ -3304,13 +3286,13 @@
         <v>190</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C44" s="20" t="s">
         <v>54</v>
       </c>
       <c r="D44" s="20" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>191</v>
@@ -3333,7 +3315,7 @@
         <v>54</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E45" s="22" t="s">
         <v>194</v>
@@ -3356,7 +3338,7 @@
         <v>54</v>
       </c>
       <c r="D46" s="20" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>197</v>
@@ -3379,7 +3361,7 @@
         <v>54</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E47" s="22" t="s">
         <v>200</v>
@@ -3388,7 +3370,7 @@
         <v>201</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3402,7 +3384,7 @@
         <v>54</v>
       </c>
       <c r="D48" s="20" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>203</v>
@@ -3425,7 +3407,7 @@
         <v>54</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E49" s="22" t="s">
         <v>206</v>
@@ -3434,7 +3416,7 @@
         <v>207</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3448,7 +3430,7 @@
         <v>54</v>
       </c>
       <c r="D50" s="20" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>209</v>
@@ -3460,60 +3442,14 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="B51" s="22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" s="23" t="s">
-        <v>54</v>
-      </c>
-      <c r="D51" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="E51" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="F51" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="G51" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C52" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="D52" s="20" t="s">
-        <v>178</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="F52" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="G52" s="20" t="s">
-        <v>48</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:G52" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A5:G50" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="3">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G6:G52">
+  <conditionalFormatting sqref="G6:G50">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Alta"</formula>
     </cfRule>
@@ -3531,7 +3467,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3544,7 +3480,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -3564,7 +3500,7 @@
     </row>
     <row r="3" spans="1:6" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="34" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="29"/>
@@ -3594,7 +3530,7 @@
     </row>
     <row r="6" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
@@ -3704,7 +3640,7 @@
     </row>
     <row r="13" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -3823,13 +3759,13 @@
         <v>107</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3843,7 +3779,7 @@
         <v>110</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>75</v>
@@ -3863,13 +3799,13 @@
         <v>113</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E21" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -3883,44 +3819,44 @@
         <v>116</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E22" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="26" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+    </row>
+    <row r="25" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B25" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C25" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D23" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="F23" s="23" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
-        <v>221</v>
-      </c>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
+      <c r="D25" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
@@ -3933,7 +3869,7 @@
         <v>122</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="E26" s="23" t="s">
         <v>75</v>
@@ -4033,7 +3969,7 @@
         <v>137</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E31" s="23" t="s">
         <v>75</v>
@@ -4042,35 +3978,35 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="s">
+    <row r="33" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="26" t="s">
+        <v>216</v>
+      </c>
+      <c r="B33" s="27"/>
+      <c r="C33" s="27"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="27"/>
+    </row>
+    <row r="34" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B34" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C34" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D34" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="E32" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="F32" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="26" t="s">
-        <v>222</v>
-      </c>
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
+      <c r="E34" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
@@ -4083,7 +4019,7 @@
         <v>143</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E35" s="23" t="s">
         <v>75</v>
@@ -4103,7 +4039,7 @@
         <v>146</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E36" s="23" t="s">
         <v>75</v>
@@ -4123,7 +4059,7 @@
         <v>149</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E37" s="23" t="s">
         <v>75</v>
@@ -4143,7 +4079,7 @@
         <v>152</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E38" s="23" t="s">
         <v>75</v>
@@ -4163,7 +4099,7 @@
         <v>155</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E39" s="23" t="s">
         <v>75</v>
@@ -4183,13 +4119,13 @@
         <v>158</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E40" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -4203,13 +4139,13 @@
         <v>161</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E41" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -4223,13 +4159,13 @@
         <v>164</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E42" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -4269,62 +4205,62 @@
         <v>75</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+    </row>
+    <row r="47" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="B45" s="22" t="s">
+      <c r="B47" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C47" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="D47" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E47" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="C45" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="D45" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E45" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="F45" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="B46" s="22" t="s">
+      <c r="F47" s="23" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="B48" s="22" t="s">
         <v>176</v>
       </c>
-      <c r="D46" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E46" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="B48" s="27"/>
-      <c r="C48" s="27"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
+      <c r="C48" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="D48" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F48" s="23" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="49" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B49" s="22" t="s">
         <v>179</v>
@@ -4333,10 +4269,10 @@
         <v>180</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>178</v>
+        <v>75</v>
       </c>
       <c r="F49" s="23" t="s">
         <v>48</v>
@@ -4353,7 +4289,7 @@
         <v>183</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E50" s="23" t="s">
         <v>75</v>
@@ -4373,7 +4309,7 @@
         <v>186</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E51" s="23" t="s">
         <v>75</v>
@@ -4393,10 +4329,10 @@
         <v>189</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E52" s="23" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="F52" s="23" t="s">
         <v>48</v>
@@ -4413,10 +4349,10 @@
         <v>192</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E53" s="23" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="F53" s="23" t="s">
         <v>48</v>
@@ -4436,7 +4372,7 @@
         <v>66</v>
       </c>
       <c r="E54" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F54" s="23" t="s">
         <v>48</v>
@@ -4456,7 +4392,7 @@
         <v>66</v>
       </c>
       <c r="E55" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F55" s="23" t="s">
         <v>48</v>
@@ -4476,10 +4412,10 @@
         <v>66</v>
       </c>
       <c r="E56" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F56" s="23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -4496,7 +4432,7 @@
         <v>66</v>
       </c>
       <c r="E57" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F57" s="23" t="s">
         <v>48</v>
@@ -4516,10 +4452,10 @@
         <v>66</v>
       </c>
       <c r="E58" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F58" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
@@ -4536,64 +4472,24 @@
         <v>66</v>
       </c>
       <c r="E59" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="F59" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="B60" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="C60" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="D60" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="E60" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="F60" s="23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="21" t="s">
-        <v>214</v>
-      </c>
-      <c r="B61" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="C61" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="D61" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="E61" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="F61" s="23" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A13:F13"/>
   </mergeCells>
-  <conditionalFormatting sqref="F6:F61">
+  <conditionalFormatting sqref="F6:F59">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Alta"</formula>
     </cfRule>

</xml_diff>